<commit_message>
Implemented Redis caching for user, organization, and dashboard
</commit_message>
<xml_diff>
--- a/Second Project/src/database/users.xlsx
+++ b/Second Project/src/database/users.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -457,9 +457,64 @@
         <v>1783870503480-Saleha_Rafique_CV.pdf</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>77095d8d-007e-45db-aa73-e18c14bcc41c</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Usman</v>
+      </c>
+      <c r="C3" t="str">
+        <v>usman12345@gmail.com</v>
+      </c>
+      <c r="D3" t="str">
+        <v>$2b$10$NjWw4dpeWXW9elDbk4ufvemrqJavtrNv1YaUDLhkGtyCGg/Wvhc4m</v>
+      </c>
+      <c r="E3" t="str">
+        <v>User</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Male</v>
+      </c>
+      <c r="G3" t="str">
+        <v>2000-01-01</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Google</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>d6589794-228b-4171-8a36-1fbc6e1ec7a3</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Usman</v>
+      </c>
+      <c r="C4" t="str">
+        <v>usman@gmail.com</v>
+      </c>
+      <c r="D4" t="str">
+        <v>$2b$10$nv1jul.zT8txZBCd0xQAv.AU4M4rLVyeC6rSo3hmyCB6mhnOi3i2q</v>
+      </c>
+      <c r="E4" t="str">
+        <v>User</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Male</v>
+      </c>
+      <c r="G4" t="str">
+        <v>2000-01-01</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Google</v>
+      </c>
+      <c r="I4" t="str">
+        <v>1784287876221-1.sql</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>